<commit_message>
middleware upgraded to proxy
</commit_message>
<xml_diff>
--- a/public/templates/customer-import-template.xlsx
+++ b/public/templates/customer-import-template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17d395c6d5503caa/Desktop/360/GenY/Home Lands/CMU/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git_geny\hl-sop\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{14178BAF-0E8F-4068-A4B4-3A219E38B7BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E89F01E-9DA5-428A-A0B9-4B0C27DB5819}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{9CA99D7B-32A6-4653-AEB0-280AC958A579}"/>
   </bookViews>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -39,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Customer Name</t>
   </si>
@@ -69,13 +67,19 @@
   </si>
   <si>
     <t>Property 3 Address</t>
+  </si>
+  <si>
+    <t>other emails</t>
+  </si>
+  <si>
+    <t>Other Telephone</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -473,14 +477,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D0F37F6-E57F-4293-AE2D-FB81E0386508}">
-  <dimension ref="A1:J12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L12"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="10" width="19.5703125" customWidth="1"/>
-    <col min="11" max="11" width="17.7109375" customWidth="1"/>
+    <col min="1" max="12" width="19.625" customWidth="1"/>
+    <col min="13" max="13" width="17.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="15">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -491,28 +495,34 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -523,8 +533,10 @@
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -535,8 +547,10 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -547,8 +561,10 @@
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -559,8 +575,10 @@
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+    </row>
+    <row r="6" spans="1:12">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -571,8 +589,10 @@
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+    </row>
+    <row r="7" spans="1:12">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -583,8 +603,10 @@
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+    </row>
+    <row r="8" spans="1:12">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -595,8 +617,10 @@
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+    </row>
+    <row r="9" spans="1:12">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -607,8 +631,10 @@
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+    </row>
+    <row r="10" spans="1:12">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -619,8 +645,10 @@
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+    </row>
+    <row r="11" spans="1:12">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -631,8 +659,10 @@
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+    </row>
+    <row r="12" spans="1:12">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -643,6 +673,8 @@
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>